<commit_message>
refactor: remove delta volume and price computations. aggregated stock changes to households at the calibration year
</commit_message>
<xml_diff>
--- a/Data_preprocessing/src/Hybridization/mappings/IOT-energy_consumers.xlsx
+++ b/Data_preprocessing/src/Hybridization/mappings/IOT-energy_consumers.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="col_label" sheetId="1" state="visible" r:id="rId2"/>
@@ -185,7 +185,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.33"/>
@@ -429,8 +429,8 @@
       <c r="B22" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="0" t="s">
-        <v>16</v>
+      <c r="C22" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -441,7 +441,7 @@
         <v>17</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -461,7 +461,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">

</xml_diff>

<commit_message>
Removed Stock Changes from the IOT for sales taxes exemption coherence with SCAF.
</commit_message>
<xml_diff>
--- a/Data_preprocessing/src/Hybridization/mappings/IOT-energy_consumers.xlsx
+++ b/Data_preprocessing/src/Hybridization/mappings/IOT-energy_consumers.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="20">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t xml:space="preserve">DELTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stock_changes</t>
   </si>
   <si>
     <t xml:space="preserve">CI_imp</t>
@@ -184,8 +181,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.33"/>
@@ -420,28 +417,6 @@
       </c>
       <c r="C21" s="1" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B23" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -461,7 +436,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -476,7 +451,7 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
@@ -487,13 +462,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>20</v>
-      </c>
       <c r="C3" s="0" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>